<commit_message>
create Job_02 and Job_03
</commit_message>
<xml_diff>
--- a/testData/JobData.xlsx
+++ b/testData/JobData.xlsx
@@ -3,14 +3,20 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="164011"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell\eclipse-workspace\PsyHire_V03\testData\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="25260" windowHeight="7230"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="11550" windowHeight="6690"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -20,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="25">
   <si>
     <t>Job title</t>
   </si>
@@ -89,6 +95,12 @@
   </si>
   <si>
     <t xml:space="preserve">Python Backend developer </t>
+  </si>
+  <si>
+    <t>ExpectedSkills</t>
+  </si>
+  <si>
+    <t>[Test Automation,Selenium WebDriver,Java,TestNG,Testing]</t>
   </si>
 </sst>
 </file>
@@ -655,4 +667,221 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:N2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="H2">
+        <v>2</v>
+      </c>
+      <c r="I2">
+        <v>2</v>
+      </c>
+      <c r="J2" t="s">
+        <v>11</v>
+      </c>
+      <c r="K2">
+        <v>700000</v>
+      </c>
+      <c r="L2">
+        <v>1000000</v>
+      </c>
+      <c r="M2" t="s">
+        <v>6</v>
+      </c>
+      <c r="N2">
+        <v>25</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:O2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="23.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.85546875" customWidth="1"/>
+    <col min="8" max="8" width="19" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="56" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="H2">
+        <v>2</v>
+      </c>
+      <c r="I2">
+        <v>2</v>
+      </c>
+      <c r="J2" t="s">
+        <v>11</v>
+      </c>
+      <c r="K2">
+        <v>700000</v>
+      </c>
+      <c r="L2">
+        <v>1000000</v>
+      </c>
+      <c r="M2" t="s">
+        <v>6</v>
+      </c>
+      <c r="N2">
+        <v>25</v>
+      </c>
+      <c r="O2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fixed Job_03, need to be updated
</commit_message>
<xml_diff>
--- a/testData/JobData.xlsx
+++ b/testData/JobData.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="11550" windowHeight="6690"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="11550" windowHeight="6690" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -100,7 +100,7 @@
     <t>ExpectedSkills</t>
   </si>
   <si>
-    <t>[Test Automation,Selenium WebDriver,Java,TestNG,Testing]</t>
+    <t>Test Automation,Selenium WebDriver,Java,TestNG,Testing</t>
   </si>
 </sst>
 </file>
@@ -859,7 +859,7 @@
         <v>2</v>
       </c>
       <c r="I2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J2" t="s">
         <v>11</v>

</xml_diff>